<commit_message>
feat(F-NAR-019): TREE-COL-015 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-015.xlsx
+++ b/stories/arbres/TREE-COL-015.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Au bout d'une rue tranquille, une petite maison ouvre ses volets sur un jardin. Aniss y vit avec papa et maman. Ce matin-là, une averse vient de laver les dalles. Les feuilles brillent, et le toit laisse tomber ses dernières gouttes. Dans la cuisine, papa coupe de la menthe pour la soupe. Maman compte les assiettes pendant que la casserole frémit. En ce moment, Aniss construit un garage près de la fenêtre. Soudain, un éclair argenté traverse la pierre dehors. On dirait une route pour une toute petite voiture ! Aniss colle son nez à la vitre. Au bout de la trace avance un escargot couleur noisette. Papa ! Maman ! Venez voir ! Mais la casserole souffle au même instant. Tu disais quelque chose, Aniss ? L'escargot ! Il va disparaître ! Dehors, l'animal disparaît derrière un pot. Un rayon de soleil glisse déjà sur les dalles. Sa route va sécher. Il faut la suivre maintenant ! Aniss attend que la casserole se taise. Merci d'avoir attendu, Aniss. Montre-nous ton secret. Nous venons avec toi. Aniss enfile ses bottes. L'enquête peut commencer.</t>
+          <t>Au bout d'une rue tranquille, une petite maison ouvre ses volets sur un jardin. Aniss y vit avec papa et maman. Ce matin-là, une averse vient de laver les dalles. Les feuilles brillent, et le toit laisse tomber ses dernières gouttes. Dans la cuisine, papa coupe de la menthe pour la soupe. Maman compte les assiettes pendant que la casserole frémit. En ce moment, Aniss construit un garage près de la fenêtre. Soudain, un éclair argenté traverse la pierre dehors. On dirait une route pour une toute petite voiture ! Aniss colle son nez à la vitre. Au bout de la trace avance un escargot couleur noisette. Papa ! Maman ! Venez voir ! Mais la casserole souffle au même instant. Tu disais quelque chose, Aniss ? L'escargot ! Il va disparaître ! Dehors, l'animal disparaît derrière un pot. Un rayon de soleil glisse déjà sur les dalles. Aniss attend que la casserole se taise. Merci d'avoir attendu, Aniss. Sa route va sécher. Il faut la suivre maintenant ! Montre-nous ton secret. Nous venons avec toi. Aniss enfile ses bottes. L'enquête peut commencer.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au bout d'une rue tranquille, une petite maison ouvre ses volets sur un jardin. Aniss y vit avec papa et maman. Ce matin-là, une averse vient de laver les dalles. Les feuilles brillent, et le toit laisse tomber ses dernières gouttes. Dans la cuisine, papa coupe de la menthe pour la soupe. Maman compte les assiettes pendant que la casserole frémit. En ce moment, Aniss construit un garage près de la fenêtre. Soudain, un éclair argenté traverse la pierre dehors. On dirait une route pour une toute petite voiture ! Aniss colle son nez à la vitre. Au bout de la trace avance un escargot couleur noisette. Papa ! Maman ! Venez voir ! Mais la casserole souffle au même instant. Tu disais quelque chose, Aniss ? L'escargot ! Il va disparaître ! Dehors, l'animal disparaît derrière un pot. Un rayon de soleil glisse déjà sur les dalles. Sa route va sécher. Il faut la suivre maintenant ! Aniss attend que la casserole se taise. Merci d'avoir attendu, Aniss. Montre-nous ton secret. Nous venons avec toi. Aniss enfile ses bottes. L'enquête peut commencer.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au bout d'une rue tranquille, une petite maison ouvre ses volets sur un jardin. Aniss y vit avec papa et maman. Ce matin-là, une averse vient de laver les dalles. Les feuilles brillent, et le toit laisse tomber ses dernières gouttes. Dans la cuisine, papa coupe de la menthe pour la soupe. Maman compte les assiettes pendant que la casserole frémit. En ce moment, Aniss construit un garage près de la fenêtre. Soudain, un éclair argenté traverse la pierre dehors. On dirait une route pour une toute petite voiture ! Aniss colle son nez à la vitre. Au bout de la trace avance un escargot couleur noisette. Papa ! Maman ! Venez voir ! Mais la casserole souffle au même instant. Tu disais quelque chose, Aniss ? L'escargot ! Il va disparaître ! Dehors, l'animal disparaît derrière un pot. Un rayon de soleil glisse déjà sur les dalles. Aniss attend que la casserole se taise. Merci d'avoir attendu, Aniss. Sa route va sécher. Il faut la suivre maintenant ! Montre-nous ton secret. Nous venons avec toi. Aniss enfile ses bottes. L'enquête peut commencer.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Au bout d'une rue tranquille, une petite maison ouvre ses volets sur un jardin. Aniss y vit avec papa et maman. Ce matin-là, une averse vient de laver les dalles. Les feuilles brillent, et le toit laisse tomber ses dernières gouttes. Dans la cuisine, papa coupe de la menthe pour la soupe. Maman compte les assiettes pendant que la casserole frémit. En ce moment, Aniss construit un garage près de la fenêtre. Soudain, un éclair argenté traverse la pierre dehors. On dirait une route pour une toute petite voiture ! Aniss colle son nez à la vitre. Au bout de la trace avance un escargot couleur noisette. Papa ! Maman ! Venez voir ! Mais la casserole souffle au même instant. Tu disais quelque chose, Aniss ? L'escargot ! Il va disparaître ! Dehors, l'animal disparaît derrière un pot. Un rayon de soleil glisse déjà sur les dalles. Sa route va sécher. Il faut la suivre maintenant ! Aniss attend que la casserole se taise. Merci d'avoir attendu, Aniss. Montre-nous ton secret. Nous venons avec toi. Aniss enfile ses bottes. L'enquête peut commencer. [pause]</t>
+          <t>Au bout d'une rue tranquille, une petite maison ouvre ses volets sur un jardin. Aniss y vit avec papa et maman. Ce matin-là, une averse vient de laver les dalles. Les feuilles brillent, et le toit laisse tomber ses dernières gouttes. Dans la cuisine, papa coupe de la menthe pour la soupe. Maman compte les assiettes pendant que la casserole frémit. En ce moment, Aniss construit un garage près de la fenêtre. Soudain, un éclair argenté traverse la pierre dehors. On dirait une route pour une toute petite voiture ! Aniss colle son nez à la vitre. Au bout de la trace avance un escargot couleur noisette. Papa ! Maman ! Venez voir ! Mais la casserole souffle au même instant. Tu disais quelque chose, Aniss ? L'escargot ! Il va disparaître ! Dehors, l'animal disparaît derrière un pot. Un rayon de soleil glisse déjà sur les dalles. Aniss attend que la casserole se taise. Merci d'avoir attendu, Aniss. Sa route va sécher. Il faut la suivre maintenant ! Montre-nous ton secret. Nous venons avec toi. Aniss enfile ses bottes. L'enquête peut commencer. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1361,10 +1361,10 @@
 enfant-m|Il va disparaître !
 narrateur|Dehors, l'animal disparaît derrière un pot.
 narrateur|Un rayon de soleil glisse déjà sur les dalles.
+narrateur|Aniss attend que la casserole se taise.
+papa|Merci d'avoir attendu, Aniss.
 enfant-m|Sa route va sécher.
 enfant-m|Il faut la suivre maintenant !
-narrateur|Aniss attend que la casserole se taise.
-papa|Merci d'avoir attendu, Aniss.
 maman|Montre-nous ton secret.
 maman|Nous venons avec toi.
 narrateur|Aniss enfile ses bottes.
@@ -17252,7 +17252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17309,6 +17309,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>